<commit_message>
Plan: three shorts per day (63) plus 4 long videos
Every short has an EN title, a UA title and a short description;
shorts are grouped by day. Formats: Motion + HeyGen and Motion.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/swan-content-plan.xlsx
+++ b/files/swan-content-plan.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="План 21 день" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План 21 день'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План 21 день'!$A$1:$K$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,18 +435,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,40 +459,50 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Слот</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Формат</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Назва (EN)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Назва (UA)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Про що</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Розділи (довгі)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Нарізка з</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Опубліковано</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Перегляди</t>
         </is>
@@ -502,843 +514,2659 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>“Home every weekend”: what's really behind it</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>«Home every weekend»: що за цим стоїть</t>
+          <t>Job Ad Autopsy #1: “Home every weekend”</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Розбір оголошення №1: «Home every weekend»</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>Розбираємо вигадане оголошення про роботу. Чому фраза «додому щовихідних» нічого не гарантує і яке одне питання треба поставити перевізнику.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Motion + HeyGen</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>5 questions that make a bad recruiter nervous</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>5 питань, від яких поганий рекрутер нервує</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>П'ять прямих питань перед підписанням: скільки водіїв пішло, зразок settlement, practical чи short милі, простій, home time письмово. Добрий рекрутер відповість на всі.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Practical miles vs short miles in 20 seconds</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Practical і short милі за 20 секунд</t>
+          <t>Dispatch Files, ep. 1: “Still good for home Friday?”</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>На карті: водій проїхав 1 000 миль, а заплатили за 940. Показуємо різницю й дві фрази, які треба спитати.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+          <t>Dispatch Files, серія 1: «Ще в силі, що додому в п'ятницю?»</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Чат із диспетчером: дім знову переносять. Типовий розвиток розмови й правильне питання про графік.</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Довге</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>How Truck Drivers Get Paid: Per Mile, Percentage, Hourly (2026)</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Як платять водіям вантажівок: за милю, відсоток, погодинно (2026)</t>
+          <t>Practical miles vs short miles in 20 seconds</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Усі моделі оплати: за милю (practical і short милі), відсоток від вантажу, погодинна й тижнева гарантія. Доплати за простій і відрахування, що питати перевізника.</t>
+          <t>Practical і short милі за 20 секунд</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Центи за милю, Відсоток, Погодинна, Гарантія, Detention, layover, stop pay, Відрахування, Settlement</t>
+          <t>На карті: водій проїхав 1 000 миль, а заплатили за 940. Показуємо різницю й дві фрази, які треба спитати.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>CAT scale: how not to be overweight</t>
+          <t>Motion + HeyGen</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>CAT scale: як не отримати перевантаження</t>
+          <t>Reply to @driver: how fast do I get paid?</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Схема осей і розподілу вантажу. Що робити, якщо вага на осях не сходиться.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>Відповідь водієві: як швидко мені заплатять?</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий відповідає на питання з коментарів: як працює графік виплат і що завжди просити в письмовому вигляді.</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Reply to @driver: how fast do I get paid?</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Відповідь водієві: як швидко мені заплатять?</t>
+          <t>CAT scale: how not to be overweight</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Ведучий відповідає на питання з коментарів: як працює графік виплат і що завжди просити в письмовому вигляді.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>CAT scale: як не отримати перевантаження</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Схема осей і розподілу вантажу. Що робити, якщо вага на осях не сходиться.</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Dispatch Files, ep. 1: “Still good for home Friday?”</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Dispatch Files, серія 1: «Ще в силі, що додому в п'ятницю?»</t>
+          <t>Where a $1,000 load really goes (example)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Чат із диспетчером: дім знову переносять. Типовий розвиток розмови й правильне питання про графік.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>Куди насправді йде вантаж на $1,000 (приклад)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Схема від вантажу до чека водія. Усі цифри підписані як приклад.</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>How truck drivers shower on the road</t>
+          <t>Motion + HeyGen</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Як водії-далекобійники миються в дорозі</t>
+          <t>Home time: the answers to listen for</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Покроково: truck stop, талон на душ, правила. Популярна тема про побут у рейсі.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+          <t>Home time: на що звертати увагу у відповідях</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий розбирає три типові відповіді про home time: що звучить конкретно, а що розмито.</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Home time: the answers to listen for</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Home time: на що звертати увагу у відповідях</t>
+          <t>How truck drivers shower on the road</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Ведучий розбирає три типові відповіді про home time: що звучить конкретно, а що розмито.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
+          <t>Як водії-далекобійники миються в дорозі</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Покроково: truck stop, талон на душ, правила. Популярна тема про побут у рейсі.</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>довге</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>Довге</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Motion + HeyGen</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>How to Switch Trucking Companies Without Losing Money</t>
-        </is>
-      </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Як змінити перевізника й не втратити гроші</t>
+          <t>How Truck Drivers Get Paid: Per Mile, Percentage, Hourly (2026)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Коли йти, що перевірити в контракті й settlement, escrow та утримання, лізинг техніки, пауза між роботами. Що вимагати від нового перевізника.</t>
+          <t>Як платять водіям вантажівок: за милю, відсоток, погодинно (2026)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Коли йти, Контракт і settlement, Escrow, Лізинг техніки, Пауза між роботами, Що питати</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>Усі моделі оплати: за милю (practical і short милі), відсоток від вантажу, погодинна й тижнева гарантія. Доплати за простій і відрахування, що питати перевізника.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Центи за милю, Відсоток, Погодинна, Гарантія, Detention, layover, stop pay, Відрахування, Settlement</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Where a $1,000 load really goes (example)</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Куди насправді йде вантаж на $1,000 (приклад)</t>
+          <t>Detention: after how many hours should you be paid?</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Схема від вантажу до чека водія. Усі цифри підписані як приклад.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+          <t>Detention: через скільки годин очікування мають платити?</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Таймер на екрані: що таке вільний час на складі й що фіксувати, щоб отримати оплату.</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>OTR vs Regional vs Local in 30 seconds</t>
+          <t>Motion + HeyGen</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>OTR, Regional і Local за 30 секунд</t>
+          <t>Why drivers leave their carrier: 5 reasons</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Карта й лічильник ночей: скільки днів удома в кожному типі роботи.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
+          <t>Чому водії залишають перевізника: 5 причин</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>П'ять причин, які називають водії: графік, гроші, диспетчер, техніка, ставлення. Короткий розбір без вигаданих історій.</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Why drivers leave their carrier: 5 reasons</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Чому водії залишають перевізника: 5 причин</t>
+          <t>Per mile or percentage: which pays more when freight is slow?</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>П'ять причин, які називають водії: графік, гроші, диспетчер, техніка, ставлення. Короткий розбір без вигаданих історій.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
+          <t>За милю чи відсоток: що платить більше, коли вантажів мало?</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Кадр із довгого відео про оплату: два графіки по тижнях і коли виграє кожна модель.</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>How much fuel does a semi hold? What a fill-up costs (example)</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Скільки пального вміщує тягач і скільки коштує заправка (приклад)</t>
+          <t>OTR vs Regional vs Local in 30 seconds</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Об'єм баків, ціна повної заправки на прикладі й чому паливо так впливає на оплату.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
+          <t>OTR, Regional і Local за 30 секунд</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Карта й лічильник ночей: скільки днів удома в кожному типі роботи.</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Detention: after how many hours should you be paid?</t>
+          <t>Motion + HeyGen</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Detention: через скільки годин очікування мають платити?</t>
+          <t>Reply to @driver: can I pick my lanes?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Таймер на екрані: що таке вільний час на складі й що фіксувати, щоб отримати оплату.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
+          <t>Відповідь водієві: чи можна обирати маршрути?</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий пояснює, як працює вибір лейнів і як про це питати перевізника.</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Довге</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Truck Driver Home Time: What “Home Weekly” Really Means</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Home time водія: що насправді означає «home weekly»</t>
+          <t>3 deductions that surprise drivers on a settlement</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>OTR, regional, local і dedicated: скільки ночей удома в кожному, як про це питати й що вимагати письмово.</t>
+          <t>3 відрахування, які дивують водіїв у settlement</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Що значить home weekly, OTR, Regional, Local, Dedicated, Що вимагати письмово</t>
+          <t>Escrow, обладнання, паливо: як вони виглядають у розрахунковому листі і що саме питати.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Reply to @driver: can I pick my lanes?</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Відповідь водієві: чи можна обирати маршрути?</t>
+          <t>How much fuel does a semi hold? What a fill-up costs (example)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Ведучий пояснює, як працює вибір лейнів і як про це питати перевізника.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
+          <t>Скільки пального вміщує тягач і скільки коштує заправка (приклад)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Об'єм баків, ціна повної заправки на прикладі й чому паливо так впливає на оплату.</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>What a DOT officer checks first</t>
+          <t>Motion + HeyGen</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Що перевіряє офіцер DOT насамперед</t>
+          <t>Thinking about leaving your carrier? Try these 3 things first</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Схема огляду: документи, ELD, стан тягача. Три речі, на які дивляться першими.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
+          <t>Думаєте піти від перевізника? Спробуйте спершу 3 речі</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Три практичні кроки перед рішенням: поговорити з диспетчером, зафіксувати проблему письмово, порівняти умови.</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Job Ad Autopsy #2: “Brand-new equipment”</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Розбір оголошення №2: «Brand-new equipment»</t>
+          <t>Job Ad Autopsy #2: “Top pay”</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Вигадане оголошення: що означає «нова техніка» і що спитати про вік тягачів і обладнання.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
+          <t>Розбір оголошення №2: «Top pay»</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Вигадане оголошення: що означає «найкраща оплата» без цифр і умов і що спитати.</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Thinking about leaving your carrier? Try these 3 things first</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Думаєте піти від перевізника? Спробуйте спершу 3 речі</t>
+          <t>What a DOT officer checks first</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Три практичні кроки перед рішенням: поговорити з диспетчером, зафіксувати проблему письмово, порівняти умови.</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
+          <t>Що перевіряє офіцер DOT насамперед</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Схема огляду: документи, ELD, стан тягача. Три речі, на які дивляться першими.</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Inside a sleeper cab: what's in it</t>
+          <t>Motion + HeyGen</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Усередині кабіни зі спальним місцем: що там є</t>
+          <t>What a trucking recruiter's day really looks like</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Ілюстрована кабіна з підписами: ліжко, холодильник, інвертор, зберігання. Для тих, хто хоче уявити побут у рейсі.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
+          <t>Яким насправді буває день рекрутера в тракінгу</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Рекрутер розповідає про свій день: дзвінки, питання водіїв, що вирішується швидко, а що ні. Без прикрас.</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Довге</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>How Truckers Live in the Cab: Sleeping, Showering, Eating</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Як водії живуть у кабіні: сон, душ, їжа</t>
+          <t>Dispatch Files, ep. 2: “The load changed again”</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Повний огляд побуту в рейсі: ліжко, душ, їжа, паркування, прання й зв'язок із родиною.</t>
+          <t>Dispatch Files, серія 2: «Вантаж знову змінили»</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Сон, Душ, Їжа, Паркування, Прання, Сім'я</t>
+          <t>Чат із диспетчером: маршрут змінюється в останню мить. Що відповісти й що зафіксувати.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Staying close to family from the road: 5 habits</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Як тримати зв'язок із сім'єю з дороги: 5 звичок</t>
+          <t>Inside a sleeper cab: what's in it</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>П'ять простих звичок, що допомагають бути поруч, коли ви в рейсі.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
+          <t>Усередині кабіни зі спальним місцем: що там є</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Ілюстрована кабіна з підписами: ліжко, холодильник, інвертор, зберігання. Для тих, хто хоче уявити побут у рейсі.</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Dispatch Files, ep. 2: “Just push through your hours”</t>
+          <t>Motion + HeyGen</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Dispatch Files, серія 2: «Просто доїдь за годинами»</t>
+          <t>Staying close to family from the road: 5 habits</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Чат із диспетчером про тиск вийти за ліміти HOS і як відповісти, не псуючи стосунки.</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr"/>
+          <t>Як тримати зв'язок із сім'єю з дороги: 5 звичок</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>П'ять простих звичок, що допомагають бути поруч, коли ви в рейсі.</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Шортс</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Motion + HeyGen</t>
+          <t>Шортс</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>What a trucking recruiter's day really looks like</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Яким насправді буває день рекрутера в тракінгу</t>
+          <t>Hours of Service in 30 seconds</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Рекрутер розповідає про свій день: дзвінки, питання водіїв, що вирішується швидко, а що ні. Без прикрас.</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr"/>
+          <t>Hours of Service за 30 секунд</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>П'ять правил FMCSA на екрані ELD: 11 годин руху, 14-годинне вікно, 30 хвилин перерви, ліміт 60/70 годин, 34-годинний рестарт.</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>довге</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Довге</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>How to Switch Trucking Companies Without Losing Money</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Як змінити перевізника й не втратити гроші</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Коли йти, що перевірити в контракті й settlement, escrow та утримання, лізинг техніки, пауза між роботами. Що вимагати від нового перевізника.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Коли йти, Контракт і settlement, Escrow, Лізинг техніки, Пауза між роботами, Що питати</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Dispatch Files, ep. 3: “Waiting 5 hours at the dock”</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Dispatch Files, серія 3: «П'ять годин чекаю на доку»</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Чат із диспетчером про довге очікування на складі і про те, коли починається оплата простою.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>What a good answer from a recruiter sounds like</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Як звучить добра відповідь рекрутера</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий порівнює дві відповіді на те саме питання: конкретну і розмиту.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>What to check in your contract before you leave a carrier</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Що перевірити в контракті, перш ніж піти від перевізника</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Кадр із довгого відео: пункти про escrow, лізинг і закриття розрахунків.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Promises vs the contract: 3 things to check in writing</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Обіцянки проти контракту: 3 пункти, які треба бачити письмово</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Спліт-екран «що сказали» і «що в документі»: home time, оплата, відрахування.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Reply to @driver: do I need experience?</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Відповідь водієві: чи потрібен досвід?</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий коротко пояснює вимоги до досвіду й що ще дивляться при відборі.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>What you can lose when you switch carriers</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Що можна втратити при зміні перевізника</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Утримані кошти, бонуси, вислуга: короткий чекліст перед звільненням.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Job Ad Autopsy #3: “Brand-new equipment”</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Розбір оголошення №3: «Brand-new equipment»</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Вигадане оголошення: що означає «нова техніка» і що спитати про вік тягачів і обладнання.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>The weekly guarantee: what counts and what doesn't</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Тижнева гарантія: що в неї входить, а що ні</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий пояснює, як рахують гарантований мінімум і що на нього не впливає.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>34-hour restart in 20 seconds</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>34-годинний рестарт за 20 секунд</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Схема на ELD: коли тиждень обнуляється і що не рахується відпочинком.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>The 30-minute break rule</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Правило 30-хвилинної перерви</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Коли її потрібно брати і що вважається перервою.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Reply to @driver: what's orientation like?</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Відповідь водієві: яка вона, орієнтація?</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий розповідає, як проходить орієнтація й що взяти з собою.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>What your ELD actually records</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Що насправді записує ваш ELD</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Іконки на екрані: час, милі, двигун, місцезнаходження.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Dispatch Files, ep. 4: “Where's my layover pay?”</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Dispatch Files, серія 4: «Де моя оплата за layover?»</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Чат із диспетчером про ніч в очікуванні вантажу і що йому писати.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Sign-on bonus: when you actually get it</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Sign-on бонус: коли його насправді виплачують</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий пояснює типові умови виплати бонусу і що уточнити письмово.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>How to check a settlement sheet in 60 seconds</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Як перевірити розрахунковий лист за 60 секунд</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Червона ручка на прикладі листа: милі, ставка, відрахування, чистий підсумок.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>довге</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Довге</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Truck Driver Home Time: What “Home Weekly” Really Means</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Home time водія: що насправді означає «home weekly»</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>OTR, regional, local і dedicated: скільки ночей удома в кожному, як про це питати й що вимагати письмово.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Що значить home weekly, OTR, Regional, Local, Dedicated, Що вимагати письмово</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Team driving: how two drivers share the clock</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Командна їзда: як двоє водіїв ділять час</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Один веде, другий відпочиває в спальнику. Як це вкладається в ліміти HOS.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Planning your time at home as a driver</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Як планувати час удома водієві</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Практичні поради: вихідні, сім'я, відпочинок і що зробити за перший вечір.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>What “home weekly” means in writing</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Що означає «home weekly» у письмовому вигляді</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Календар на 4 тижні й слова, які варто бачити в умовах.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Dedicated: what it is and who it fits</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Dedicated: що це і кому підходить</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Схема постійного маршруту й чим він відрізняється від OTR.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Reply to @driver: what if I want to leave?</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Відповідь водієві: що якщо я захочу піти?</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий пояснює, як працює розрахунок і що вирішують письмово.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Nights at home per month: three job types</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Ночі вдома за місяць: три типи роботи</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Лічильник ночей для OTR, regional і local.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Job Ad Autopsy #4: “Sign-on bonus*”</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Розбір оголошення №4: «Sign-on bonus*»</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Вигадане оголошення із зірочкою й дрібним шрифтом: що там зазвичай приховано.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Truck stop rules nobody explains</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Правила truck stop, які ніхто не пояснює</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Паркування, душ, черга на ваги й етикет, про які не пишуть в інструкціях.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>What happens at a shipper, step by step</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Що відбувається на складі відправника, крок за кроком</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Двір, ворота, док, чек-ін, пломба: схема на графіці.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>A 14-hour driving day, hour by hour</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>14-годинний робочий день водія, година за годиною</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Таймлайн HOS: 11 годин руху, 14-годинне вікно, перерва.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>The question that tells you how a carrier treats drivers</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Питання, яке показує, як перевізник ставиться до водіїв</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>«Скільки водіїв пішло за останні 90 днів?» і як сприймати відповідь.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>5 things to check on a truck before you roll</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>5 речей перевірити на тягачі перед виїздом</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Чекліст: шини, гальма, світло, зчіпка, рівні рідин.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Dispatch Files, ep. 5: “Just push through your hours”</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Dispatch Files, серія 5: «Просто доїдь за годинами»</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Чат із диспетчером про тиск вийти за ліміти HOS і як відповісти, не псуючи стосунки.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Reply to @driver: what happens if the truck breaks down?</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Відповідь водієві: що буде, якщо тягач зламався?</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий пояснює, куди дзвонити, як фіксувати час і що з оплатою.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>How drivers sleep in a sleeper cab</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Як водії сплять у кабіні зі спальним місцем</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Схема ліжка, штор і температури, що допомагає виспатися в рейсі.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>довге</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Довге</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>How Truckers Live in the Cab: Sleeping, Showering, Eating</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Як водії живуть у кабіні: сон, душ, їжа</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Повний огляд побуту в рейсі: ліжко, душ, їжа, паркування, прання й зв'язок із родиною.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Сон, Душ, Їжа, Паркування, Прання, Сім'я</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>APU, inverter, fridge: what each one does</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>APU, інвертор, холодильник: що це і навіщо</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Іконки на ілюстрованій кабіні й для чого кожен пристрій.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Pets on the truck: what to know</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Тварини в кабіні: що треба знати</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий розповідає про правила й домовленості щодо тварин.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>5 easy meals you can make in a cab</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>5 простих страв, які можна приготувати в кабіні</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Рецепти на інвертор і міні-кухню.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Winter: 7 things to keep in your cab</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Зима: 7 речей, які мають бути в кабіні</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Чекліст: ланцюги, обігрів, їжа, вода, ліхтар.</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Can family ride along? What to know</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Чи можна їхати з сім'єю? Що треба знати</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий пояснює, як вирішується питання пасажирів у кабіні.</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Where to park when the truck stop is full</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Де паркуватися, коли truck stop заповнений</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Схема варіантів: rest area, склад, запасні стоянки.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Job Ad Autopsy #5: “Home time varies”</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Розбір оголошення №5: «Home time varies»</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Вигадане оголошення: що ховається за словами «home time varies» і що вимагати письмово.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Motion + HeyGen</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Your first paycheck at a new carrier: what to expect and when</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Ваш перший чек у нового перевізника: чого чекати і коли</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Ведучий пояснює типовий графік виплат і що перевірити в розрахунковому листі.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Шортс</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>What is a reefer trailer?</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Що таке reefer-причіп?</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Схема: холодильна установка, температурний режим, пальне для неї.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:K68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add news channel tab, fix funnel wording, update plan
Two main tabs: Swan Transportation and the news channel (concept and
first-week plan, 11 shorts + weekly roundup). Funnel last step renamed,
data collection date shown, orientation topic replaced.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/swan-content-plan.xlsx
+++ b/files/swan-content-plan.xlsx
@@ -1953,17 +1953,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Reply to @driver: what's orientation like?</t>
+          <t>Reply to @driver: how does getting started work?</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Відповідь водієві: яка вона, орієнтація?</t>
+          <t>Відповідь водієві: як проходить старт роботи?</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Ведучий розповідає, як проходить орієнтація й що взяти з собою.</t>
+          <t>Ведучий розповідає, як виглядає початок співпраці й що підготувати заздалегідь.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>

</xml_diff>